<commit_message>
Remove redundant sections from weekly tracker
- Drop duplicated reward menu, weekly levels, and per-day bank deposit
  table from the tracker page (those live on dedicated pages)
- Simplify Weekly Summary to just 3 fields: total, level, bank deposit
- Add links to Reward Shop and Quick Reference pages
- PDF/XLSX page 2 keeps rewards + levels for standalone printout value

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/public/weekly-tracker.xlsx
+++ b/docs/public/weekly-tracker.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="77">
   <si>
     <t>Quest Mode — Weekly Tracker</t>
   </si>
@@ -110,34 +110,16 @@
     <t>Weekly Summary</t>
   </si>
   <si>
-    <t>Total Earned</t>
-  </si>
-  <si>
-    <t>Total Deductions</t>
-  </si>
-  <si>
-    <t>Weekly Total (earned − deductions)</t>
+    <t>Weekly Total (sum of daily totals)</t>
   </si>
   <si>
     <t>Weekly Level</t>
   </si>
   <si>
-    <t>Bank Deposit (half of gross, round up)</t>
-  </si>
-  <si>
-    <t>Day</t>
-  </si>
-  <si>
-    <t>Gross Earned</t>
-  </si>
-  <si>
-    <t>Bank Deposit</t>
-  </si>
-  <si>
-    <t>Week Total</t>
-  </si>
-  <si>
-    <t>Bank Before: _____ + Deposits: _____ − Spent: _____ = Bank After: _____</t>
+    <t>Bank Deposit (half of total, round up)</t>
+  </si>
+  <si>
+    <t>Bank: Before _____ + Deposit _____ − Spent _____ = After _____</t>
   </si>
   <si>
     <t>Reward Shop</t>
@@ -267,7 +249,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -299,15 +281,6 @@
       <b/>
       <color rgb="FF22C55E"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
     </font>
     <font>
       <sz val="10"/>
@@ -397,7 +370,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -415,20 +388,16 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -448,7 +417,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -791,7 +760,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1498,143 +1467,25 @@
       </c>
       <c r="C30" s="8"/>
     </row>
-    <row r="31" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C31" s="8"/>
-    </row>
-    <row r="33" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B33" s="9"/>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="35" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="36" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C36" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="37" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C37" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="38" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="39" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C39" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="40" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C40" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="42" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C42" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="B44" s="13"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
-      <c r="F44" s="13"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="7">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A32:F32"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1657,204 +1508,204 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>44</v>
+      <c r="A3" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="15" t="s">
+      <c r="A8" s="12" t="s">
         <v>44</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>44</v>
+      <c r="A16" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="C24" s="17"/>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="20" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
+      <c r="B25" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="C25" s="19"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="20" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="23" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="18" t="s">
+      <c r="B26" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
+      <c r="C26" s="21"/>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B27" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="C24" s="19"/>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="20" t="s">
+      <c r="C27" s="23"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B28" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="C25" s="21"/>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="22" t="s">
+      <c r="C28" s="25"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="B26" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="C26" s="23"/>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="B27" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="C27" s="25"/>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="B28" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="C28" s="27"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="28"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B31"/>
       <c r="C31"/>

</xml_diff>

<commit_message>
Expand deductions section and add starting balance
- List all 5 deduction behaviors in the score sheet instead of blank lines
- Add deductions reference table to page 2 of PDF and sheet 2 of XLSX
- Replace "Bank Before/After" with "Starting Balance / New Balance"
- Keep one blank deduction row for custom entries

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/public/weekly-tracker.xlsx
+++ b/docs/public/weekly-tracker.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="94">
   <si>
     <t>Quest Mode — Weekly Tracker</t>
   </si>
@@ -104,6 +104,21 @@
     <t>Deductions (max −8/day)</t>
   </si>
   <si>
+    <t>Clip yellow (−2) / orange (−4) / red (−6)</t>
+  </si>
+  <si>
+    <t>Not listening after 2 asks (−1)</t>
+  </si>
+  <si>
+    <t>Screaming or tantrum (−2)</t>
+  </si>
+  <si>
+    <t>Disrespectful language (−2)</t>
+  </si>
+  <si>
+    <t>Lying (−3)</t>
+  </si>
+  <si>
     <t>Daily Total</t>
   </si>
   <si>
@@ -119,7 +134,7 @@
     <t>Bank Deposit (half of total, round up)</t>
   </si>
   <si>
-    <t>Bank: Before _____ + Deposit _____ − Spent _____ = After _____</t>
+    <t>Starting Balance: _____ + Deposit _____ − Spent _____ = New Balance _____</t>
   </si>
   <si>
     <t>Reward Shop</t>
@@ -237,6 +252,42 @@
   </si>
   <si>
     <t>RED</t>
+  </si>
+  <si>
+    <t>Deductions</t>
+  </si>
+  <si>
+    <t>Damage</t>
+  </si>
+  <si>
+    <t>Clip yellow / orange / red</t>
+  </si>
+  <si>
+    <t>−2 / −4 / −6</t>
+  </si>
+  <si>
+    <t>Not listening after 2 asks</t>
+  </si>
+  <si>
+    <t>−1</t>
+  </si>
+  <si>
+    <t>Screaming or tantrum</t>
+  </si>
+  <si>
+    <t>−2</t>
+  </si>
+  <si>
+    <t>Disrespectful language</t>
+  </si>
+  <si>
+    <t>Lying</t>
+  </si>
+  <si>
+    <t>−3</t>
+  </si>
+  <si>
+    <t>Max −8/day. Earned points are never removed.</t>
   </si>
   <si>
     <t>Protected Activities (always safe)</t>
@@ -249,7 +300,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -298,6 +349,10 @@
       <b/>
       <color rgb="FF22C55E"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="9">
@@ -370,7 +425,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -417,6 +472,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -760,7 +817,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1376,116 +1433,261 @@
     </row>
     <row r="24" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H26" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I24" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H25" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-    </row>
-    <row r="28" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" s="8"/>
-    </row>
-    <row r="29" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
-        <v>33</v>
-      </c>
       <c r="B29" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C29" s="8"/>
-    </row>
-    <row r="30" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
-        <v>34</v>
+      <c r="C29" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H29" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="B30" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C30" s="8"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
+      <c r="C30" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I30" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" s="8"/>
+    </row>
+    <row r="34" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" s="8"/>
+    </row>
+    <row r="35" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" s="8"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="11"/>
+      <c r="C37" s="11"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="A37:F37"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1497,7 +1699,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1508,7 +1710,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1516,135 +1718,135 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B23" s="16"/>
       <c r="C23" s="16"/>
@@ -1652,67 +1854,131 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C24" s="17"/>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C25" s="19"/>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C26" s="21"/>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="22" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C27" s="23"/>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="24" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B28" s="25" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C28" s="25"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>76</v>
-      </c>
-      <c r="B31"/>
-      <c r="C31"/>
-      <c r="D31"/>
+    <row r="31" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="B38" s="27"/>
+      <c r="C38" s="27"/>
+      <c r="D38" s="27"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>93</v>
+      </c>
+      <c r="B41"/>
+      <c r="C41"/>
+      <c r="D41"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="B24:C24"/>
@@ -1720,8 +1986,10 @@
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
-    <mergeCell ref="A30:D30"/>
     <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A41:D41"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Align Quest Mode language with coaching guidance
</commit_message>
<xml_diff>
--- a/docs/public/weekly-tracker.xlsx
+++ b/docs/public/weekly-tracker.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="89">
   <si>
     <t>Quest Mode — Weekly Tracker</t>
   </si>
@@ -110,15 +110,9 @@
     <t>Not listening after 2 asks (−1)</t>
   </si>
   <si>
-    <t>Screaming or tantrum (−2)</t>
-  </si>
-  <si>
     <t>Disrespectful language (−2)</t>
   </si>
   <si>
-    <t>Lying (−3)</t>
-  </si>
-  <si>
     <t>Daily Total</t>
   </si>
   <si>
@@ -272,19 +266,10 @@
     <t>−1</t>
   </si>
   <si>
-    <t>Screaming or tantrum</t>
+    <t>Disrespectful language</t>
   </si>
   <si>
     <t>−2</t>
-  </si>
-  <si>
-    <t>Disrespectful language</t>
-  </si>
-  <si>
-    <t>Lying</t>
-  </si>
-  <si>
-    <t>−3</t>
   </si>
   <si>
     <t>Max −8/day. Earned points are never removed.</t>
@@ -817,7 +802,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1520,127 +1505,87 @@
     </row>
     <row r="27" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H27" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I27" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="28" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
+      <c r="B28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H28" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I28" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F29" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G29" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H29" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I29" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="5" t="s">
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+    </row>
+    <row r="31" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B30" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G30" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H30" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I30" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="9" t="s">
+      <c r="B31" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31" s="8"/>
+    </row>
+    <row r="32" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="9"/>
-      <c r="C32" s="9"/>
-      <c r="D32" s="9"/>
+      <c r="B32" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" s="8"/>
     </row>
     <row r="33" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
@@ -1651,43 +1596,25 @@
       </c>
       <c r="C33" s="8"/>
     </row>
-    <row r="34" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C34" s="8"/>
-    </row>
-    <row r="35" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C35" s="8"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="B37" s="11"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A35:F35"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1699,7 +1626,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1710,7 +1637,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1718,135 +1645,135 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B23" s="16"/>
       <c r="C23" s="16"/>
@@ -1854,52 +1781,52 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C24" s="17"/>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C25" s="19"/>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C26" s="21"/>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="22" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C27" s="23"/>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="24" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B28" s="25" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C28" s="25"/>
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B31" s="16"/>
       <c r="C31" s="16"/>
@@ -1910,72 +1837,56 @@
         <v>2</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B36" s="27"/>
+      <c r="C36" s="27"/>
+      <c r="D36" s="27"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="28" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="36" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="6" t="s">
+      <c r="B38" s="28"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="28"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>88</v>
       </c>
-      <c r="B36" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="37" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="27" t="s">
-        <v>91</v>
-      </c>
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="B40" s="28"/>
-      <c r="C40" s="28"/>
-      <c r="D40" s="28"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>93</v>
-      </c>
-      <c r="B41"/>
-      <c r="C41"/>
-      <c r="D41"/>
+      <c r="B39"/>
+      <c r="C39"/>
+      <c r="D39"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -1987,9 +1898,9 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A36:D36"/>
     <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A39:D39"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Rebrand to Valor and rename skills
</commit_message>
<xml_diff>
--- a/docs/public/weekly-tracker.xlsx
+++ b/docs/public/weekly-tracker.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="89">
   <si>
-    <t>Quest Mode — Weekly Tracker</t>
+    <t>Valor — Weekly Tracker</t>
   </si>
   <si>
     <t>Week of: _________________</t>
@@ -101,7 +101,7 @@
     <t>______________________</t>
   </si>
   <si>
-    <t>Deductions (max −8/day)</t>
+    <t>Dips (max −8/day)</t>
   </si>
   <si>
     <t>Clip yellow (−2) / orange (−4) / red (−6)</t>
@@ -113,25 +113,25 @@
     <t>Disrespectful language (−2)</t>
   </si>
   <si>
-    <t>Daily Total</t>
+    <t>Daily Valor</t>
   </si>
   <si>
     <t>Weekly Summary</t>
   </si>
   <si>
-    <t>Weekly Total (sum of daily totals)</t>
-  </si>
-  <si>
-    <t>Weekly Level</t>
-  </si>
-  <si>
-    <t>Bank Deposit (half of total, round up)</t>
-  </si>
-  <si>
-    <t>Starting Balance: _____ + Deposit _____ − Spent _____ = New Balance _____</t>
-  </si>
-  <si>
-    <t>Reward Shop</t>
+    <t>Valor Standing (sum of daily totals)</t>
+  </si>
+  <si>
+    <t>Weekly Rank</t>
+  </si>
+  <si>
+    <t>Vault Deposit (half of total, round up)</t>
+  </si>
+  <si>
+    <t>Vault Balance: _____ + Deposit _____ − Redeemed _____ = New Balance _____</t>
+  </si>
+  <si>
+    <t>Reward List</t>
   </si>
   <si>
     <t>Weekday (Mon–Fri)</t>
@@ -143,7 +143,7 @@
     <t>Extra 30 min screen time</t>
   </si>
   <si>
-    <t>10 XP</t>
+    <t>10 Valor</t>
   </si>
   <si>
     <t>Small treat (candy, snack)</t>
@@ -152,7 +152,7 @@
     <t>Stay up 20 min past bedtime</t>
   </si>
   <si>
-    <t>15 XP</t>
+    <t>15 Valor</t>
   </si>
   <si>
     <t>Weekend (Sat–Sun)</t>
@@ -161,7 +161,7 @@
     <t>Boba or special drink</t>
   </si>
   <si>
-    <t>20 XP</t>
+    <t>20 Valor</t>
   </si>
   <si>
     <t>Pick the family movie</t>
@@ -170,13 +170,13 @@
     <t>Extra 1 hour screen time</t>
   </si>
   <si>
-    <t>25 XP</t>
+    <t>25 Valor</t>
   </si>
   <si>
     <t>Pick dinner for the family</t>
   </si>
   <si>
-    <t>30 XP</t>
+    <t>30 Valor</t>
   </si>
   <si>
     <t>Stay up 30 min past bedtime</t>
@@ -185,7 +185,7 @@
     <t>Disney trip (3–4 hours)</t>
   </si>
   <si>
-    <t>40 XP</t>
+    <t>40 Valor</t>
   </si>
   <si>
     <t>Save-Up (anytime)</t>
@@ -194,64 +194,64 @@
     <t>Small toy or book (under $15)</t>
   </si>
   <si>
-    <t>50 XP</t>
+    <t>50 Valor</t>
   </si>
   <si>
     <t>Special outing (1:1 with parent)</t>
   </si>
   <si>
-    <t>60 XP</t>
+    <t>60 Valor</t>
   </si>
   <si>
     <t>Big reward (new game, experience)</t>
   </si>
   <si>
-    <t>100 XP</t>
+    <t>100 Valor</t>
   </si>
   <si>
     <t>Nintendo Switch 2</t>
   </si>
   <si>
-    <t>250 XP</t>
-  </si>
-  <si>
-    <t>Weekly Levels</t>
-  </si>
-  <si>
-    <t>Points</t>
-  </si>
-  <si>
-    <t>Level</t>
+    <t>250 Valor</t>
+  </si>
+  <si>
+    <t>Weekly Ranks</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>Rank</t>
   </si>
   <si>
     <t>80+</t>
   </si>
   <si>
-    <t>GOLD</t>
+    <t>LEGEND</t>
   </si>
   <si>
     <t>60–79</t>
   </si>
   <si>
-    <t>GREEN</t>
+    <t>CHAMPION</t>
   </si>
   <si>
     <t>40–59</t>
   </si>
   <si>
-    <t>YELLOW</t>
+    <t>KNIGHT</t>
   </si>
   <si>
     <t>Below 40</t>
   </si>
   <si>
-    <t>RED</t>
-  </si>
-  <si>
-    <t>Deductions</t>
-  </si>
-  <si>
-    <t>Damage</t>
+    <t>RECRUIT</t>
+  </si>
+  <si>
+    <t>Dips</t>
+  </si>
+  <si>
+    <t>Dip</t>
   </si>
   <si>
     <t>Clip yellow / orange / red</t>
@@ -272,7 +272,7 @@
     <t>−2</t>
   </si>
   <si>
-    <t>Max −8/day. Earned points are never removed.</t>
+    <t>Max −8/day. Earned valor is never removed.</t>
   </si>
   <si>
     <t>Protected Activities (always safe)</t>

</xml_diff>

<commit_message>
Adopt Valor Points (VP) wording
</commit_message>
<xml_diff>
--- a/docs/public/weekly-tracker.xlsx
+++ b/docs/public/weekly-tracker.xlsx
@@ -113,7 +113,7 @@
     <t>Disrespectful language (−2)</t>
   </si>
   <si>
-    <t>Daily Valor</t>
+    <t>Daily VP</t>
   </si>
   <si>
     <t>Weekly Summary</t>
@@ -143,7 +143,7 @@
     <t>Extra 30 min screen time</t>
   </si>
   <si>
-    <t>10 Valor</t>
+    <t>10 VP</t>
   </si>
   <si>
     <t>Small treat (candy, snack)</t>
@@ -152,7 +152,7 @@
     <t>Stay up 20 min past bedtime</t>
   </si>
   <si>
-    <t>15 Valor</t>
+    <t>15 VP</t>
   </si>
   <si>
     <t>Weekend (Sat–Sun)</t>
@@ -161,7 +161,7 @@
     <t>Boba or special drink</t>
   </si>
   <si>
-    <t>20 Valor</t>
+    <t>20 VP</t>
   </si>
   <si>
     <t>Pick the family movie</t>
@@ -170,13 +170,13 @@
     <t>Extra 1 hour screen time</t>
   </si>
   <si>
-    <t>25 Valor</t>
+    <t>25 VP</t>
   </si>
   <si>
     <t>Pick dinner for the family</t>
   </si>
   <si>
-    <t>30 Valor</t>
+    <t>30 VP</t>
   </si>
   <si>
     <t>Stay up 30 min past bedtime</t>
@@ -185,7 +185,7 @@
     <t>Disney trip (3–4 hours)</t>
   </si>
   <si>
-    <t>40 Valor</t>
+    <t>40 VP</t>
   </si>
   <si>
     <t>Save-Up (anytime)</t>
@@ -194,31 +194,31 @@
     <t>Small toy or book (under $15)</t>
   </si>
   <si>
-    <t>50 Valor</t>
+    <t>50 VP</t>
   </si>
   <si>
     <t>Special outing (1:1 with parent)</t>
   </si>
   <si>
-    <t>60 Valor</t>
+    <t>60 VP</t>
   </si>
   <si>
     <t>Big reward (new game, experience)</t>
   </si>
   <si>
-    <t>100 Valor</t>
+    <t>100 VP</t>
   </si>
   <si>
     <t>Nintendo Switch 2</t>
   </si>
   <si>
-    <t>250 Valor</t>
+    <t>250 VP</t>
   </si>
   <si>
     <t>Weekly Ranks</t>
   </si>
   <si>
-    <t>Valor</t>
+    <t>VP</t>
   </si>
   <si>
     <t>Rank</t>
@@ -272,7 +272,7 @@
     <t>−2</t>
   </si>
   <si>
-    <t>Max −8/day. Earned valor is never removed.</t>
+    <t>Max −8/day. Earned VP is never removed.</t>
   </si>
   <si>
     <t>Protected Activities (always safe)</t>

</xml_diff>